<commit_message>
Add NuGet support files for TuplesAndDeconstruction project
- Created project.assets.json to manage package dependencies.
- Added TuplesAndDeconstruction.csproj.nuget.g.props and TuplesAndDeconstruction.csproj.nuget.g.targets for NuGet build properties and targets.
- Introduced project.nuget.cache to cache NuGet restore results.
</commit_message>
<xml_diff>
--- a/02.ROAD MAP/01.dotnet_roadmap.xlsx
+++ b/02.ROAD MAP/01.dotnet_roadmap.xlsx
@@ -3283,7 +3283,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="10" ht="39.75" spans="1:5">
+    <row r="10" ht="46" customHeight="1" spans="1:5">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -3414,7 +3414,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="3" ht="39.75" spans="1:5">
+    <row r="3" ht="26.5" spans="1:5">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -3448,7 +3448,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" ht="39.75" spans="1:5">
+    <row r="5" ht="26.5" spans="1:5">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -3482,7 +3482,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" ht="39.75" spans="1:5">
+    <row r="7" ht="26.5" spans="1:5">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -3516,7 +3516,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" ht="39.75" spans="1:5">
+    <row r="9" ht="26.5" spans="1:5">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -3533,7 +3533,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" ht="39.75" spans="1:5">
+    <row r="10" ht="26.5" spans="1:5">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -3564,21 +3564,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultColWidth="8.67826086956522" defaultRowHeight="14.4" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="51.8869565217391" defaultRowHeight="50" customHeight="1" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="32" customWidth="1"/>
-    <col min="3" max="3" width="45" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="1" max="1" width="3.11304347826087" customWidth="1"/>
+    <col min="2" max="2" width="21.3391304347826" customWidth="1"/>
+    <col min="3" max="3" width="51.8869565217391" customWidth="1"/>
+    <col min="4" max="4" width="12.5130434782609" customWidth="1"/>
+    <col min="5" max="5" width="15.3217391304348" customWidth="1"/>
+    <col min="6" max="16384" width="51.8869565217391" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1" spans="1:5">
+    <row r="1" customHeight="1" spans="1:5">
       <c r="A1" s="38" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="2" ht="25.5" customHeight="1" spans="1:5">
+    <row r="2" customHeight="1" spans="1:5">
       <c r="A2" s="39" t="s">
         <v>2</v>
       </c>
@@ -3595,7 +3596,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="3" ht="21.75" customHeight="1" spans="1:5">
+    <row r="3" customHeight="1" spans="1:5">
       <c r="A3" s="7">
         <v>1</v>
       </c>
@@ -3612,7 +3613,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" ht="21.75" customHeight="1" spans="1:5">
+    <row r="4" customHeight="1" spans="1:5">
       <c r="A4" s="7">
         <v>2</v>
       </c>
@@ -3629,7 +3630,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" ht="21.75" customHeight="1" spans="1:5">
+    <row r="5" customHeight="1" spans="1:5">
       <c r="A5" s="7">
         <v>3</v>
       </c>
@@ -3646,7 +3647,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" ht="21.75" customHeight="1" spans="1:5">
+    <row r="6" customHeight="1" spans="1:5">
       <c r="A6" s="7">
         <v>4</v>
       </c>
@@ -3663,7 +3664,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="7" ht="21.75" customHeight="1" spans="1:5">
+    <row r="7" customHeight="1" spans="1:5">
       <c r="A7" s="7">
         <v>5</v>
       </c>
@@ -3680,7 +3681,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" ht="21.75" customHeight="1" spans="1:5">
+    <row r="8" customHeight="1" spans="1:5">
       <c r="A8" s="7">
         <v>6</v>
       </c>
@@ -3697,7 +3698,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" ht="21.75" customHeight="1" spans="1:5">
+    <row r="9" customHeight="1" spans="1:5">
       <c r="A9" s="7">
         <v>7</v>
       </c>
@@ -3714,7 +3715,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" ht="21.75" customHeight="1" spans="1:5">
+    <row r="10" customHeight="1" spans="1:5">
       <c r="A10" s="7">
         <v>8</v>
       </c>
@@ -3731,7 +3732,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="11" ht="21.75" customHeight="1" spans="1:5">
+    <row r="11" customHeight="1" spans="1:5">
       <c r="A11" s="7">
         <v>9</v>
       </c>
@@ -3748,7 +3749,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="12" ht="21.75" customHeight="1" spans="1:5">
+    <row r="12" customHeight="1" spans="1:5">
       <c r="A12" s="7">
         <v>10</v>
       </c>
@@ -3810,7 +3811,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="3" ht="21.75" customHeight="1" spans="1:5">
+    <row r="3" ht="39.75" spans="1:5">
       <c r="A3" s="9">
         <v>1</v>
       </c>
@@ -3827,7 +3828,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" ht="21.75" customHeight="1" spans="1:5">
+    <row r="4" ht="53" spans="1:5">
       <c r="A4" s="9">
         <v>2</v>
       </c>
@@ -3844,7 +3845,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" ht="21.75" customHeight="1" spans="1:5">
+    <row r="5" ht="39.75" spans="1:5">
       <c r="A5" s="9">
         <v>3</v>
       </c>
@@ -3861,7 +3862,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" ht="21.75" customHeight="1" spans="1:5">
+    <row r="6" ht="39.75" spans="1:5">
       <c r="A6" s="9">
         <v>4</v>
       </c>
@@ -3878,7 +3879,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" ht="21.75" customHeight="1" spans="1:5">
+    <row r="7" ht="39.75" spans="1:5">
       <c r="A7" s="9">
         <v>5</v>
       </c>
@@ -3895,7 +3896,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="8" ht="21.75" customHeight="1" spans="1:5">
+    <row r="8" ht="39.75" spans="1:5">
       <c r="A8" s="9">
         <v>6</v>
       </c>
@@ -3912,7 +3913,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" ht="21.75" customHeight="1" spans="1:5">
+    <row r="9" ht="39.75" spans="1:5">
       <c r="A9" s="9">
         <v>7</v>
       </c>
@@ -3929,7 +3930,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="10" ht="21.75" customHeight="1" spans="1:5">
+    <row r="10" ht="39.75" spans="1:5">
       <c r="A10" s="9">
         <v>8</v>
       </c>
@@ -3946,7 +3947,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="11" ht="21.75" customHeight="1" spans="1:5">
+    <row r="11" ht="26.5" spans="1:5">
       <c r="A11" s="9">
         <v>9</v>
       </c>
@@ -4008,7 +4009,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="3" ht="21.75" customHeight="1" spans="1:5">
+    <row r="3" ht="39.75" spans="1:5">
       <c r="A3" s="11">
         <v>1</v>
       </c>
@@ -4025,7 +4026,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" ht="21.75" customHeight="1" spans="1:5">
+    <row r="4" ht="26.5" spans="1:5">
       <c r="A4" s="11">
         <v>2</v>
       </c>
@@ -4042,7 +4043,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" ht="21.75" customHeight="1" spans="1:5">
+    <row r="5" ht="39.75" spans="1:5">
       <c r="A5" s="11">
         <v>3</v>
       </c>
@@ -4059,7 +4060,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" ht="21.75" customHeight="1" spans="1:5">
+    <row r="6" ht="39.75" spans="1:5">
       <c r="A6" s="11">
         <v>4</v>
       </c>
@@ -4076,7 +4077,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" ht="21.75" customHeight="1" spans="1:5">
+    <row r="7" ht="39.75" spans="1:5">
       <c r="A7" s="11">
         <v>5</v>
       </c>
@@ -4093,7 +4094,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" ht="21.75" customHeight="1" spans="1:5">
+    <row r="8" ht="39.75" spans="1:5">
       <c r="A8" s="11">
         <v>6</v>
       </c>
@@ -4110,7 +4111,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" ht="21.75" customHeight="1" spans="1:5">
+    <row r="9" ht="39.75" spans="1:5">
       <c r="A9" s="11">
         <v>7</v>
       </c>
@@ -4127,7 +4128,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" ht="21.75" customHeight="1" spans="1:5">
+    <row r="10" ht="39.75" spans="1:5">
       <c r="A10" s="11">
         <v>8</v>
       </c>
@@ -4144,7 +4145,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="11" ht="21.75" customHeight="1" spans="1:5">
+    <row r="11" ht="39.75" spans="1:5">
       <c r="A11" s="11">
         <v>9</v>
       </c>
@@ -4161,7 +4162,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="12" ht="21.75" customHeight="1" spans="1:5">
+    <row r="12" ht="39.75" spans="1:5">
       <c r="A12" s="11">
         <v>10</v>
       </c>

</xml_diff>